<commit_message>
Updating download_sivep and data
</commit_message>
<xml_diff>
--- a/output/tb_desc_rr_2021-05-17.xlsx
+++ b/output/tb_desc_rr_2021-05-17.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -389,22 +389,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>14198 (9020-18769)</t>
+          <t>14202 (9021-18774)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>22354 (18259-33322)</t>
+          <t>22358 (18266-33329)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>17764 (15333-19234)</t>
+          <t>17768 (15338-19244)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>28894 (22596-37648)</t>
+          <t>28900 (22598-37659)</t>
         </is>
       </c>
     </row>
@@ -416,56 +416,56 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>21282</t>
+          <t>21290</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>52529</t>
+          <t>52540</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>22237</t>
+          <t>22241</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>52529</t>
+          <t>52540</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Admissions, n(%) [n = 1,149,141]</t>
+          <t>Admissions, n(%) [n = 1,149,406]</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>468,021 (100.0%)</t>
+          <t>468,123 (100.0%)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>681,120 (100.0%)</t>
+          <t>681,283 (100.0%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>170,042 (100.0%)</t>
+          <t>170,086 (100.0%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>511,078 (100.0%)</t>
+          <t>511,197 (100.0%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sex, n (%) [n = 1,148,955]</t>
+          <t>Sex, n (%) [n = 1,149,220]</t>
         </is>
       </c>
     </row>
@@ -477,22 +477,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>205,307 (43.9%)</t>
+          <t>205,345 (43.9%)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>305,072 (44.8%)</t>
+          <t>305,142 (44.8%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>75,717 (44.5%)</t>
+          <t>75,735 (44.5%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>229,355 (44.9%)</t>
+          <t>229,407 (44.9%)</t>
         </is>
       </c>
     </row>
@@ -504,29 +504,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>262,645 (56.1%)</t>
+          <t>262,709 (56.1%)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>375,931 (55.2%)</t>
+          <t>376,024 (55.2%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>94,291 (55.5%)</t>
+          <t>94,317 (55.5%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>281,640 (55.1%)</t>
+          <t>281,707 (55.1%)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Age, median (IQR) [n = 1,149,141]</t>
+          <t>Age, median (IQR) [n = 1,149,406]</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -553,88 +553,88 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>20-39 years, n(%) [n = 1,149,141]</t>
+          <t>20-39 years, n(%) [n = 1,149,406]</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>61,422 (13.1%)</t>
+          <t>61,440 (13.1%)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>86,132 (12.6%)</t>
+          <t>86,153 (12.6%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>18,594 (10.9%)</t>
+          <t>18,597 (10.9%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>67,538 (13.2%)</t>
+          <t>67,556 (13.2%)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>40-59 years [n = 1,149,141]</t>
+          <t>40-59 years [n = 1,149,406]</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>153,163 (32.7%)</t>
+          <t>153,199 (32.7%)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>240,589 (35.3%)</t>
+          <t>240,649 (35.3%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>53,623 (31.5%)</t>
+          <t>53,637 (31.5%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>186,966 (36.6%)</t>
+          <t>187,012 (36.6%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>&gt;=60 years [n = 1,149,141]</t>
+          <t>&gt;=60 years [n = 1,149,406]</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>253,436 (54.2%)</t>
+          <t>253,484 (54.1%)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>354,399 (52.0%)</t>
+          <t>354,481 (52.0%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>97,825 (57.5%)</t>
+          <t>97,852 (57.5%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>256,574 (50.2%)</t>
+          <t>256,629 (50.2%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Self-reported race, n(%) [n = 922,421]</t>
+          <t>Self-reported race, n(%) [n = 922,639]</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>6,258 (1.1%)</t>
+          <t>6,259 (1.1%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>4,613 (1.1%)</t>
+          <t>4,614 (1.1%)</t>
         </is>
       </c>
     </row>
@@ -673,22 +673,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>183,714 (51.3%)</t>
+          <t>183,757 (51.3%)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>246,765 (43.7%)</t>
+          <t>246,829 (43.7%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>58,749 (41.9%)</t>
+          <t>58,761 (41.9%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>188,016 (44.3%)</t>
+          <t>188,068 (44.3%)</t>
         </is>
       </c>
     </row>
@@ -727,29 +727,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>168,007 (46.9%)</t>
+          <t>168,043 (46.9%)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>310,161 (55.0%)</t>
+          <t>310,235 (55.0%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>79,402 (56.7%)</t>
+          <t>79,425 (56.7%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>230,759 (54.4%)</t>
+          <t>230,810 (54.4%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Self-reported level of education, n (%) [n = 409,492]</t>
+          <t>Self-reported level of education, n (%) [n = 409,592]</t>
         </is>
       </c>
     </row>
@@ -761,22 +761,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>25,540 (15.4%)</t>
+          <t>25,547 (15.4%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>39,874 (16.4%)</t>
+          <t>39,884 (16.4%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>11,694 (19.0%)</t>
+          <t>11,699 (19.0%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>28,180 (15.5%)</t>
+          <t>28,185 (15.5%)</t>
         </is>
       </c>
     </row>
@@ -788,22 +788,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>51,958 (31.2%)</t>
+          <t>51,968 (31.2%)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>78,185 (32.2%)</t>
+          <t>78,208 (32.2%)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>19,213 (31.2%)</t>
+          <t>19,218 (31.2%)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>58,972 (32.5%)</t>
+          <t>58,990 (32.5%)</t>
         </is>
       </c>
     </row>
@@ -815,22 +815,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>12,452 (7.5%)</t>
+          <t>12,453 (7.5%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>13,763 (5.7%)</t>
+          <t>13,767 (5.7%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>3,493 (5.7%)</t>
+          <t>3,496 (5.7%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10,270 (5.7%)</t>
+          <t>10,271 (5.7%)</t>
         </is>
       </c>
     </row>
@@ -842,515 +842,542 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>76,356 (45.9%)</t>
+          <t>76,374 (45.9%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>111,364 (45.8%)</t>
+          <t>111,391 (45.8%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>27,106 (44.1%)</t>
+          <t>27,111 (44.1%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>84,258 (46.4%)</t>
+          <t>84,280 (46.4%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Area of residence, n(%) [n = 1,018,408]</t>
+          <t>IS_CAPITAL [n = 1,149,406]</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>225,815 (48.2%)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>256,900 (37.7%)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>71,103 (41.8%)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>185,797 (36.3%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Peri-urban</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>1,444 (0.3%)</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1,969 (0.3%)</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>535 (0.4%)</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>1,434 (0.3%)</t>
+          <t>Area of residence, n(%) [n = 1,018,644]</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Peri-urban</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>17,318 (4.2%)</t>
+          <t>1,444 (0.3%)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>28,297 (4.7%)</t>
+          <t>1,969 (0.3%)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>6,024 (4.0%)</t>
+          <t>535 (0.4%)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>22,273 (4.9%)</t>
+          <t>1,434 (0.3%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>396,936 (95.5%)</t>
+          <t>17,321 (4.2%)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>572,444 (95.0%)</t>
+          <t>28,298 (4.7%)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>143,873 (95.6%)</t>
+          <t>6,024 (4.0%)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>428,571 (94.8%)</t>
+          <t>22,274 (4.9%)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Hypoxaemia, n (%) [n = 972,582]</t>
+          <t>Urban</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>272,793 (69.5%)</t>
+          <t>397,028 (95.5%)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>455,703 (78.6%)</t>
+          <t>572,584 (95.0%)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>104,780 (72.9%)</t>
+          <t>143,911 (95.6%)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>350,923 (80.4%)</t>
+          <t>428,673 (94.8%)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ICU admission, n (%) [n = 1,026,454]</t>
+          <t>Hypoxaemia, n (%) [n = 972,803]</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>156,550 (37.6%)</t>
+          <t>272,853 (69.5%)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>228,966 (37.5%)</t>
+          <t>455,803 (78.6%)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>59,645 (38.7%)</t>
+          <t>104,801 (72.9%)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>169,321 (37.1%)</t>
+          <t>351,002 (80.4%)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Total Respiratory Support, n(%) [n = 993,651]</t>
+          <t>ICU admission, n (%) [n = 1,026,693]</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>291,119 (73.2%)</t>
+          <t>156,588 (37.6%)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>496,814 (83.3%)</t>
+          <t>229,015 (37.5%)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>115,290 (77.7%)</t>
+          <t>59,660 (38.7%)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>381,524 (85.2%)</t>
+          <t>169,355 (37.1%)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>NIV, n (%) [n = 993,651]</t>
+          <t>Total Respiratory Support, n(%) [n = 993,880]</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>207,306 (52.2%)</t>
+          <t>291,188 (73.2%)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>365,152 (61.2%)</t>
+          <t>496,927 (83.3%)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>87,617 (59.0%)</t>
+          <t>115,317 (77.7%)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>277,535 (62.0%)</t>
+          <t>381,610 (85.2%)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>IMV, n (%) [n = 993,651]</t>
+          <t>NIV, n (%) [n = 993,880]</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>83,813 (21.1%)</t>
+          <t>207,352 (52.2%)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>131,662 (22.1%)</t>
+          <t>365,236 (61.2%)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>27,673 (18.6%)</t>
+          <t>87,637 (59.0%)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>103,989 (23.2%)</t>
+          <t>277,599 (62.0%)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>IMV inside ICU, n(%) [n = 210,420]</t>
+          <t>IMV, n (%) [n = 993,880]</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>70,658 (86.5%)</t>
+          <t>83,836 (21.1%)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>110,417 (85.8%)</t>
+          <t>131,691 (22.1%)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>23,860 (87.9%)</t>
+          <t>27,680 (18.6%)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>86,557 (85.2%)</t>
+          <t>104,011 (23.2%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>IMV outside ICU, n(%) [n = 210,420]</t>
+          <t>IMV inside ICU, n(%) [n = 210,471]</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>11,044 (13.5%)</t>
+          <t>70,679 (86.5%)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>18,301 (14.2%)</t>
+          <t>110,438 (85.8%)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>3,271 (12.1%)</t>
+          <t>23,865 (87.9%)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>15,030 (14.8%)</t>
+          <t>86,573 (85.2%)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Admissions with an outcome, n(%) [n = 1,149,141]</t>
+          <t>IMV outside ICU, n(%) [n = 210,471]</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>435,751 (93.1%)</t>
+          <t>11,046 (13.5%)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>579,279 (85.0%)</t>
+          <t>18,308 (14.2%)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>153,093 (90.0%)</t>
+          <t>3,273 (12.1%)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>426,186 (83.4%)</t>
+          <t>15,035 (14.8%)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Overall, n (%) [n = 1,015,030]</t>
+          <t>Admissions with an outcome, n(%) [n = 1,149,406]</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>155,405 (35.7%)</t>
+          <t>435,852 (93.1%)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>226,013 (39.0%)</t>
+          <t>579,417 (85.0%)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>50,715 (33.1%)</t>
+          <t>153,131 (90.0%)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>175,298 (41.1%)</t>
+          <t>426,286 (83.4%)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>20-39 years [n = 127,362]</t>
+          <t>Overall, n (%) [n = 1,015,269]</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>6,532 (11.6%)</t>
+          <t>155,430 (35.7%)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>12,052 (17.0%)</t>
+          <t>226,075 (39.0%)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1,852 (11.2%)</t>
+          <t>50,730 (33.1%)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>10,200 (18.7%)</t>
+          <t>175,345 (41.1%)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>40-59 years [n = 341,642]</t>
+          <t>20-39 years [n = 127,391]</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>30,874 (21.8%)</t>
+          <t>6,533 (11.6%)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>54,960 (27.5%)</t>
+          <t>12,055 (17.0%)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>9,155 (19.1%)</t>
+          <t>1,852 (11.2%)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>45,805 (30.1%)</t>
+          <t>10,203 (18.7%)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>&gt;= 60 years [n = 546,026]</t>
+          <t>40-59 years [n = 341,727]</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>117,999 (49.6%)</t>
+          <t>30,880 (21.8%)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>159,001 (51.6%)</t>
+          <t>54,976 (27.5%)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>39,708 (44.7%)</t>
+          <t>9,158 (19.1%)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>119,293 (54.3%)</t>
+          <t>45,818 (30.1%)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ICU admission, n (%) [n = 349,934]</t>
+          <t>&gt;= 60 years [n = 546,151]</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>85,692 (57.8%)</t>
+          <t>118,017 (49.6%)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>130,944 (64.9%)</t>
+          <t>159,044 (51.6%)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>30,626 (56.1%)</t>
+          <t>39,720 (44.7%)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>100,318 (68.2%)</t>
+          <t>119,324 (54.3%)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>NIV, n (%) [n = 498,841]</t>
+          <t>ICU admission, n (%) [n = 350,019]</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>51,954 (26.9%)</t>
+          <t>85,711 (57.8%)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>85,580 (28.0%)</t>
+          <t>130,973 (64.9%)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>19,542 (24.8%)</t>
+          <t>30,633 (56.1%)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>66,038 (29.1%)</t>
+          <t>100,340 (68.2%)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>IMV, n (%) [n = 201,643]</t>
+          <t>NIV, n (%) [n = 498,956]</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>64,157 (79.2%)</t>
+          <t>51,958 (26.9%)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>100,494 (83.3%)</t>
+          <t>85,603 (28.0%)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>20,761 (78.9%)</t>
+          <t>19,547 (24.9%)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>79,733 (84.5%)</t>
+          <t>66,056 (29.1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>IMV, n (%) [n = 201,696]</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>64,175 (79.2%)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>100,520 (83.3%)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>20,767 (78.9%)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>79,753 (84.5%)</t>
         </is>
       </c>
     </row>

</xml_diff>